<commit_message>
feat(creditos/reportes): capital no determinable, causas de incompletitud, UF explicada, rango vs corte
- Capital sin desglose: «No determinable: sin desglose» en vez de 0; capital
  confirmado, sin desglose y por conciliar contiguos y destacados; columna de
  determinacion. Exclusion de las tres categorias comprobada en prueba; no se suman.
- Totales con todas las causas de informacion incompleta y su conteo.
- UF: unidades, pares USD-CLP y UF-CLP con fecha y fuente (ufPorFecha) y ejemplo
  con la division que cuadra al centavo.
- Pantalla, Excel y PDF: el rango filtra movimientos, el corte determina saldos;
  subtotales rotulados «cartera al corte» o «solo filas del rango».
- Aviso de descarga limitada a empresas autorizadas para perfiles «ver».
- Sin cambios en creditos.js. jest 37, e2e 89, ejemplos 46.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WWmFk3cyaXSqjsmvoCZymx
</commit_message>
<xml_diff>
--- a/docs/ejemplos/creditos-reportes/frisku-sin-tc.xlsx
+++ b/docs/ejemplos/creditos-reportes/frisku-sin-tc.xlsx
@@ -9,15 +9,15 @@
     <sheet sheetId="3" name="Cuotas y pagos" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Resumen'!$14:$14</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Créditos'!$14:$14</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Resumen'!$16:$16</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Créditos'!$16:$16</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="90">
   <si>
     <t>Créditos · Frisku Foods</t>
   </si>
@@ -43,6 +43,12 @@
     <t>sin rango · todas las cuotas y pagos</t>
   </si>
   <si>
+    <t>Cómo leer</t>
+  </si>
+  <si>
+    <t>La fecha de corte determina los SALDOS (capital, sin desglose, intereses, vencido, por conciliar, pagado) de toda la cartera filtrada. El rango solo filtra los MOVIMIENTOS listados (cuotas por vencimiento, pagos por fecha efectiva) y no cambia ningún saldo. Los totales marcados «cartera al corte» incluyen todo el crédito; los marcados «solo filas del rango», únicamente las filas listadas.</t>
+  </si>
+  <si>
     <t>Empresa (deudora)</t>
   </si>
   <si>
@@ -70,7 +76,10 @@
     <t>todos · solo pagos vigentes (los anulados no se listan)</t>
   </si>
   <si>
-    <t>⚠ Sin tipo de cambio a la fecha de corte (los totales en USD están INCOMPLETOS; estos importes siguen en su moneda original): crédito D (N° 4) · Frisku Foods · Banco Perú Demo · PEN.</t>
+    <t>⚠ Sin tipo de cambio al corte (los totales en USD no los incluyen; siguen en su moneda original): crédito D (N° 4) · Frisku Foods · Banco Perú Demo · PEN.</t>
+  </si>
+  <si>
+    <t>Resumen · saldos al corte de toda la cartera filtrada (cartera al corte; el rango no los cambia)</t>
   </si>
   <si>
     <t>Empresa</t>
@@ -85,10 +94,13 @@
     <t>Créditos</t>
   </si>
   <si>
-    <t>Capital pendiente (confirmado)</t>
-  </si>
-  <si>
-    <t>Sin desglose pendiente</t>
+    <t>Capital pendiente confirmado</t>
+  </si>
+  <si>
+    <t>Sin desglose (capital no determinable)</t>
+  </si>
+  <si>
+    <t>Por conciliar (no confirmado)</t>
   </si>
   <si>
     <t>Intereses pendientes</t>
@@ -97,24 +109,27 @@
     <t>Cargos pendientes</t>
   </si>
   <si>
-    <t>Pendiente total</t>
+    <t>Pendiente total confirmado (capital + sin desglose + intereses + cargos)</t>
   </si>
   <si>
     <t>Vencido</t>
   </si>
   <si>
-    <t>Por conciliar (no confirmado)</t>
-  </si>
-  <si>
     <t>Pagado al corte</t>
   </si>
   <si>
-    <t>Capital pendiente USD</t>
+    <t>Capital confirmado USD</t>
+  </si>
+  <si>
+    <t>Sin desglose USD</t>
   </si>
   <si>
     <t>Por conciliar USD</t>
   </si>
   <si>
+    <t>Advertencias (información incompleta)</t>
+  </si>
+  <si>
     <t>Línea a línea</t>
   </si>
   <si>
@@ -124,10 +139,13 @@
     <t>sin TC</t>
   </si>
   <si>
-    <t>Total Frisku Foods · PEN</t>
-  </si>
-  <si>
-    <t>Total Frisku Foods en USD (INCOMPLETO: falta TC)</t>
+    <t>sin tipo de cambio al corte (1)</t>
+  </si>
+  <si>
+    <t>Total Frisku Foods · PEN · cartera al corte (INCOMPLETO: ver advertencias)</t>
+  </si>
+  <si>
+    <t>Total Frisku Foods en USD · cartera al corte (INCOMPLETO: ver advertencias)</t>
   </si>
   <si>
     <t>USD</t>
@@ -136,6 +154,9 @@
     <t>Detalle de créditos · generado 13-10-2026 (ejemplo)</t>
   </si>
   <si>
+    <t>Créditos · saldos al corte de todo el crédito (cartera al corte)</t>
+  </si>
+  <si>
     <t>ID crédito</t>
   </si>
   <si>
@@ -154,66 +175,78 @@
     <t>Vencimiento final</t>
   </si>
   <si>
+    <t>Determinación del capital</t>
+  </si>
+  <si>
+    <t>Pendiente total confirmado</t>
+  </si>
+  <si>
+    <t>Pagos al corte</t>
+  </si>
+  <si>
+    <t>Cuotas en rango</t>
+  </si>
+  <si>
+    <t>Estado</t>
+  </si>
+  <si>
+    <t>TC al corte (unidades por 1 US$)</t>
+  </si>
+  <si>
+    <t>Advertencias</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>Banco Perú Demo</t>
+  </si>
+  <si>
+    <t>Capital de trabajo</t>
+  </si>
+  <si>
+    <t>Determinado</t>
+  </si>
+  <si>
+    <t>Vigente</t>
+  </si>
+  <si>
+    <t>SIN TC</t>
+  </si>
+  <si>
+    <t>sin tipo de cambio al corte</t>
+  </si>
+  <si>
+    <t>Subtotal Frisku Foods · PEN · cartera al corte (todo el crédito, no solo el rango)</t>
+  </si>
+  <si>
+    <t>Detalle de cuotas (por vencimiento) y pagos registrados (por fecha efectiva) · generado 13-10-2026 (ejemplo)</t>
+  </si>
+  <si>
+    <t>Cuotas · movimientos listados (solo filas del rango); estado al corte</t>
+  </si>
+  <si>
+    <t>ID cuota</t>
+  </si>
+  <si>
+    <t>Vencimiento</t>
+  </si>
+  <si>
+    <t>Origen</t>
+  </si>
+  <si>
+    <t>Capital</t>
+  </si>
+  <si>
+    <t>Interés</t>
+  </si>
+  <si>
+    <t>Cargos</t>
+  </si>
+  <si>
     <t>Sin desglose</t>
   </si>
   <si>
-    <t>Por conciliar</t>
-  </si>
-  <si>
-    <t>Pagos al corte</t>
-  </si>
-  <si>
-    <t>Cuotas en rango</t>
-  </si>
-  <si>
-    <t>Estado</t>
-  </si>
-  <si>
-    <t>TC (moneda por US$)</t>
-  </si>
-  <si>
-    <t>D</t>
-  </si>
-  <si>
-    <t>Banco Perú Demo</t>
-  </si>
-  <si>
-    <t>Capital de trabajo</t>
-  </si>
-  <si>
-    <t>Vigente</t>
-  </si>
-  <si>
-    <t>SIN TC</t>
-  </si>
-  <si>
-    <t>Subtotal Frisku Foods · PEN</t>
-  </si>
-  <si>
-    <t>Detalle de cuotas (por vencimiento) y pagos registrados (por fecha efectiva) · generado 13-10-2026 (ejemplo)</t>
-  </si>
-  <si>
-    <t>Cuotas</t>
-  </si>
-  <si>
-    <t>ID cuota</t>
-  </si>
-  <si>
-    <t>Vencimiento</t>
-  </si>
-  <si>
-    <t>Origen</t>
-  </si>
-  <si>
-    <t>Capital</t>
-  </si>
-  <si>
-    <t>Interés</t>
-  </si>
-  <si>
-    <t>Cargos</t>
-  </si>
-  <si>
     <t>Total cuota</t>
   </si>
   <si>
@@ -235,7 +268,10 @@
     <t>D@2027-07-01</t>
   </si>
   <si>
-    <t>Pagos registrados</t>
+    <t>Subtotal Frisku Foods · PEN · solo filas del rango</t>
+  </si>
+  <si>
+    <t>Pagos registrados · movimientos listados (solo filas del rango)</t>
   </si>
   <si>
     <t>ID pago</t>
@@ -291,6 +327,11 @@
     </font>
     <font>
       <b/>
+      <color rgb="FF0F766E"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b/>
       <color rgb="FFFFFFFF"/>
       <sz val="9"/>
     </font>
@@ -299,16 +340,11 @@
       <sz val="9"/>
     </font>
     <font>
-      <b/>
-      <color rgb="FF0F766E"/>
-      <sz val="11"/>
-    </font>
-    <font>
       <i/>
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -322,7 +358,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFB45309"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFCCFBF1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -366,7 +412,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -374,19 +420,36 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="4" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="7" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="4" fontId="7" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="8" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="8" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="4" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="8" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -862,14 +925,15 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:P20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="8" customWidth="1"/>
-    <col min="5" max="14" width="16" customWidth="1"/>
+    <col min="5" max="15" width="16" customWidth="1"/>
+    <col min="16" max="16" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
@@ -882,7 +946,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" ht="6" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" ht="6" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -897,6 +961,8 @@
       <c r="L3" s="3"/>
       <c r="M3" s="3"/>
       <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
@@ -951,192 +1017,235 @@
         <v>14</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="14" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
+      <c r="C12" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B14" s="7" t="s">
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="7" t="s">
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="D14" s="7" t="s">
+    </row>
+    <row r="16" ht="30" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A16" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="B16" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="C16" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="G14" s="7" t="s">
+      <c r="D16" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="H14" s="7" t="s">
+      <c r="E16" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="I14" s="7" t="s">
+      <c r="F16" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="J14" s="7" t="s">
+      <c r="G16" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="K14" s="7" t="s">
+      <c r="H16" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="L14" s="7" t="s">
+      <c r="I16" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="M14" s="7" t="s">
+      <c r="J16" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="N14" s="7" t="s">
+      <c r="K16" s="8" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="8"/>
-      <c r="H15" s="8"/>
-      <c r="I15" s="8"/>
-      <c r="J15" s="8"/>
-      <c r="K15" s="8"/>
-      <c r="L15" s="8"/>
-      <c r="M15" s="8"/>
-      <c r="N15" s="8"/>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B16" s="5" t="s">
+      <c r="L16" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="M16" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="D16" s="9">
-        <v>1</v>
-      </c>
-      <c r="E16" s="10">
-        <v>300000</v>
-      </c>
-      <c r="F16" s="10">
-        <v>0</v>
-      </c>
-      <c r="G16" s="10">
-        <v>33458.34</v>
-      </c>
-      <c r="H16" s="10">
-        <v>0</v>
-      </c>
-      <c r="I16" s="10">
-        <v>333458.34</v>
-      </c>
-      <c r="J16" s="10">
-        <v>0</v>
-      </c>
-      <c r="K16" s="10">
-        <v>0</v>
-      </c>
-      <c r="L16" s="10">
-        <v>0</v>
-      </c>
-      <c r="M16" s="5" t="s">
+      <c r="N16" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="N16" s="5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="11" t="s">
+      <c r="O16" s="9" t="s">
         <v>35</v>
       </c>
+      <c r="P16" s="8" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A17" s="10" t="s">
+        <v>11</v>
+      </c>
       <c r="B17" s="11"/>
-      <c r="C17" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="D17" s="12">
-        <v>1</v>
-      </c>
-      <c r="E17" s="13">
-        <v>300000</v>
-      </c>
-      <c r="F17" s="13">
-        <v>0</v>
-      </c>
-      <c r="G17" s="13">
-        <v>33458.34</v>
-      </c>
-      <c r="H17" s="13">
-        <v>0</v>
-      </c>
-      <c r="I17" s="13">
-        <v>333458.34</v>
-      </c>
-      <c r="J17" s="13">
-        <v>0</v>
-      </c>
-      <c r="K17" s="13">
-        <v>0</v>
-      </c>
-      <c r="L17" s="13">
-        <v>0</v>
-      </c>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="11"/>
+      <c r="J17" s="11"/>
+      <c r="K17" s="11"/>
+      <c r="L17" s="11"/>
       <c r="M17" s="11"/>
       <c r="N17" s="11"/>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11" t="s">
+      <c r="O17" s="11"/>
+      <c r="P17" s="10"/>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A18" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B18" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11"/>
-      <c r="H18" s="11"/>
-      <c r="I18" s="11"/>
-      <c r="J18" s="11"/>
-      <c r="K18" s="11"/>
-      <c r="L18" s="11"/>
-      <c r="M18" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="N18" s="11" t="s">
-        <v>34</v>
+      <c r="C18" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D18" s="13">
+        <v>1</v>
+      </c>
+      <c r="E18" s="14">
+        <v>300000</v>
+      </c>
+      <c r="F18" s="14">
+        <v>0</v>
+      </c>
+      <c r="G18" s="14">
+        <v>0</v>
+      </c>
+      <c r="H18" s="15">
+        <v>33458.34</v>
+      </c>
+      <c r="I18" s="15">
+        <v>0</v>
+      </c>
+      <c r="J18" s="15">
+        <v>333458.34</v>
+      </c>
+      <c r="K18" s="15">
+        <v>0</v>
+      </c>
+      <c r="L18" s="15">
+        <v>0</v>
+      </c>
+      <c r="M18" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="N18" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="O18" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="P18" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A19" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="B19" s="18"/>
+      <c r="C19" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="D19" s="19">
+        <v>1</v>
+      </c>
+      <c r="E19" s="20">
+        <v>300000</v>
+      </c>
+      <c r="F19" s="20">
+        <v>0</v>
+      </c>
+      <c r="G19" s="20">
+        <v>0</v>
+      </c>
+      <c r="H19" s="20">
+        <v>33458.34</v>
+      </c>
+      <c r="I19" s="20">
+        <v>0</v>
+      </c>
+      <c r="J19" s="20">
+        <v>333458.34</v>
+      </c>
+      <c r="K19" s="20">
+        <v>0</v>
+      </c>
+      <c r="L19" s="20">
+        <v>0</v>
+      </c>
+      <c r="M19" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="N19" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="O19" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="P19" s="17" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A20" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" s="18"/>
+      <c r="C20" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="D20" s="18"/>
+      <c r="E20" s="18"/>
+      <c r="F20" s="18"/>
+      <c r="G20" s="18"/>
+      <c r="H20" s="18"/>
+      <c r="I20" s="18"/>
+      <c r="J20" s="18"/>
+      <c r="K20" s="18"/>
+      <c r="L20" s="18"/>
+      <c r="M20" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="N20" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="O20" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="P20" s="17" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A14:N18"/>
+  <autoFilter ref="A16:P20"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
   <headerFooter>
@@ -1151,7 +1260,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:V16"/>
+  <dimension ref="A1:X18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1162,10 +1271,13 @@
     <col min="6" max="7" width="12" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
     <col min="9" max="10" width="11" customWidth="1"/>
-    <col min="11" max="17" width="16" customWidth="1"/>
-    <col min="18" max="19" width="8" customWidth="1"/>
-    <col min="20" max="21" width="22" customWidth="1"/>
-    <col min="22" max="22" width="16" customWidth="1"/>
+    <col min="11" max="13" width="16" customWidth="1"/>
+    <col min="14" max="14" width="12" customWidth="1"/>
+    <col min="15" max="18" width="16" customWidth="1"/>
+    <col min="19" max="20" width="8" customWidth="1"/>
+    <col min="21" max="22" width="22" customWidth="1"/>
+    <col min="23" max="23" width="16" customWidth="1"/>
+    <col min="24" max="24" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
@@ -1175,10 +1287,10 @@
     </row>
     <row r="2" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C2" s="2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="3" ht="6" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" ht="6" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -1201,6 +1313,8 @@
       <c r="T3" s="3"/>
       <c r="U3" s="3"/>
       <c r="V3" s="3"/>
+      <c r="W3" s="3"/>
+      <c r="X3" s="3"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
@@ -1255,204 +1369,235 @@
         <v>14</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="14" ht="30" customHeight="1" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
+      <c r="C12" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A16" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="H16" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I16" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="J16" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="K16" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="L16" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M16" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="N16" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="O16" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="P16" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q16" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="R16" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="S16" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="T16" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="U16" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="V16" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="W16" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="X16" s="8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B17" s="13">
+        <v>4</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="H17" s="15">
+        <v>300000</v>
+      </c>
+      <c r="I17" s="21">
+        <v>46204</v>
+      </c>
+      <c r="J17" s="21">
+        <v>46569</v>
+      </c>
+      <c r="K17" s="14">
+        <v>300000</v>
+      </c>
+      <c r="L17" s="14">
+        <v>0</v>
+      </c>
+      <c r="M17" s="14">
+        <v>0</v>
+      </c>
+      <c r="N17" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="O17" s="15">
+        <v>33458.34</v>
+      </c>
+      <c r="P17" s="15">
+        <v>333458.34</v>
+      </c>
+      <c r="Q17" s="15">
+        <v>0</v>
+      </c>
+      <c r="R17" s="15">
+        <v>0</v>
+      </c>
+      <c r="S17" s="13">
+        <v>0</v>
+      </c>
+      <c r="T17" s="13">
+        <v>2</v>
+      </c>
+      <c r="U17" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="V17" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="W17" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="X17" s="12" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A18" s="22"/>
+      <c r="B18" s="22"/>
+      <c r="C18" s="23" t="s">
+        <v>66</v>
+      </c>
+      <c r="D18" s="22"/>
+      <c r="E18" s="22"/>
+      <c r="F18" s="22"/>
+      <c r="G18" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="H18" s="24">
+        <v>300000</v>
+      </c>
+      <c r="I18" s="22"/>
+      <c r="J18" s="22"/>
+      <c r="K18" s="24">
+        <v>300000</v>
+      </c>
+      <c r="L18" s="24">
+        <v>0</v>
+      </c>
+      <c r="M18" s="24">
+        <v>0</v>
+      </c>
+      <c r="N18" s="22" t="s">
+        <v>62</v>
+      </c>
+      <c r="O18" s="24">
+        <v>33458.34</v>
+      </c>
+      <c r="P18" s="24">
+        <v>333458.34</v>
+      </c>
+      <c r="Q18" s="24">
+        <v>0</v>
+      </c>
+      <c r="R18" s="24">
+        <v>0</v>
+      </c>
+      <c r="S18" s="22"/>
+      <c r="T18" s="22"/>
+      <c r="U18" s="22"/>
+      <c r="V18" s="22"/>
+      <c r="W18" s="22"/>
+      <c r="X18" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="C14" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="G14" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="H14" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="I14" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="J14" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="K14" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="L14" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="M14" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="N14" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="O14" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="P14" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="Q14" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="R14" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="S14" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="T14" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="U14" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="V14" s="7" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="B15" s="9">
-        <v>4</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H15" s="10">
-        <v>300000</v>
-      </c>
-      <c r="I15" s="14">
-        <v>46204</v>
-      </c>
-      <c r="J15" s="14">
-        <v>46569</v>
-      </c>
-      <c r="K15" s="10">
-        <v>300000</v>
-      </c>
-      <c r="L15" s="10">
-        <v>0</v>
-      </c>
-      <c r="M15" s="10">
-        <v>33458.34</v>
-      </c>
-      <c r="N15" s="10">
-        <v>333458.34</v>
-      </c>
-      <c r="O15" s="10">
-        <v>0</v>
-      </c>
-      <c r="P15" s="10">
-        <v>0</v>
-      </c>
-      <c r="Q15" s="10">
-        <v>0</v>
-      </c>
-      <c r="R15" s="9">
-        <v>0</v>
-      </c>
-      <c r="S15" s="9">
-        <v>2</v>
-      </c>
-      <c r="T15" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="U15" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="V15" s="5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A16" s="15"/>
-      <c r="B16" s="15"/>
-      <c r="C16" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="15"/>
-      <c r="G16" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="H16" s="16">
-        <v>300000</v>
-      </c>
-      <c r="I16" s="15"/>
-      <c r="J16" s="15"/>
-      <c r="K16" s="16">
-        <v>300000</v>
-      </c>
-      <c r="L16" s="16">
-        <v>0</v>
-      </c>
-      <c r="M16" s="16">
-        <v>33458.34</v>
-      </c>
-      <c r="N16" s="16">
-        <v>333458.34</v>
-      </c>
-      <c r="O16" s="16">
-        <v>0</v>
-      </c>
-      <c r="P16" s="16">
-        <v>0</v>
-      </c>
-      <c r="Q16" s="16">
-        <v>0</v>
-      </c>
-      <c r="R16" s="15"/>
-      <c r="S16" s="15"/>
-      <c r="T16" s="15"/>
-      <c r="U16" s="15"/>
-      <c r="V16" s="15"/>
     </row>
   </sheetData>
-  <autoFilter ref="A14:V16"/>
+  <autoFilter ref="A16:X18"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
   <headerFooter>
@@ -1467,7 +1612,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O22"/>
+  <dimension ref="A1:O23"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -1484,7 +1629,7 @@
     </row>
     <row r="2" ht="18" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C2" s="2" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" ht="6" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
@@ -1557,255 +1702,263 @@
         <v>14</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" s="17" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="C12" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="D15" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="G15" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="H15" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="I15" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="J15" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="K15" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="L15" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="M15" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="N15" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="O15" s="7" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="B16" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="C16" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="F16" s="14">
-        <v>46388</v>
-      </c>
-      <c r="G16" s="5" t="s">
+    </row>
+    <row r="16" ht="30" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B16" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="H16" s="10">
-        <v>0</v>
-      </c>
-      <c r="I16" s="10">
-        <v>16866.67</v>
-      </c>
-      <c r="J16" s="10">
-        <v>0</v>
-      </c>
-      <c r="K16" s="10">
-        <v>0</v>
-      </c>
-      <c r="L16" s="10">
-        <v>16866.67</v>
-      </c>
-      <c r="M16" s="10">
-        <v>0</v>
-      </c>
-      <c r="N16" s="10">
-        <v>16866.67</v>
-      </c>
-      <c r="O16" s="5" t="s">
+      <c r="C16" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="F16" s="8" t="s">
         <v>70</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="H16" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="I16" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="J16" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="K16" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="L16" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="M16" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="N16" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="O16" s="8" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>9</v>
+        <v>79</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>11</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="F17" s="14">
+        <v>38</v>
+      </c>
+      <c r="F17" s="21">
+        <v>46388</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="H17" s="15">
+        <v>0</v>
+      </c>
+      <c r="I17" s="15">
+        <v>16866.67</v>
+      </c>
+      <c r="J17" s="15">
+        <v>0</v>
+      </c>
+      <c r="K17" s="15">
+        <v>0</v>
+      </c>
+      <c r="L17" s="15">
+        <v>16866.67</v>
+      </c>
+      <c r="M17" s="15">
+        <v>0</v>
+      </c>
+      <c r="N17" s="15">
+        <v>16866.67</v>
+      </c>
+      <c r="O17" s="5" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F18" s="21">
         <v>46569</v>
       </c>
-      <c r="G17" s="5" t="s">
+      <c r="G18" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="H18" s="15">
+        <v>300000</v>
+      </c>
+      <c r="I18" s="15">
+        <v>16591.67</v>
+      </c>
+      <c r="J18" s="15">
+        <v>0</v>
+      </c>
+      <c r="K18" s="15">
+        <v>0</v>
+      </c>
+      <c r="L18" s="15">
+        <v>316591.67</v>
+      </c>
+      <c r="M18" s="15">
+        <v>0</v>
+      </c>
+      <c r="N18" s="15">
+        <v>316591.67</v>
+      </c>
+      <c r="O18" s="5" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19" s="22"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="D19" s="22"/>
+      <c r="E19" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="F19" s="22"/>
+      <c r="G19" s="22"/>
+      <c r="H19" s="24">
+        <v>300000</v>
+      </c>
+      <c r="I19" s="24">
+        <v>33458.34</v>
+      </c>
+      <c r="J19" s="24">
+        <v>0</v>
+      </c>
+      <c r="K19" s="24">
+        <v>0</v>
+      </c>
+      <c r="L19" s="24">
+        <v>333458.34</v>
+      </c>
+      <c r="M19" s="24">
+        <v>0</v>
+      </c>
+      <c r="N19" s="24">
+        <v>333458.34</v>
+      </c>
+      <c r="O19" s="22"/>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="7" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A22" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C22" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="H17" s="10">
-        <v>300000</v>
-      </c>
-      <c r="I17" s="10">
-        <v>16591.67</v>
-      </c>
-      <c r="J17" s="10">
-        <v>0</v>
-      </c>
-      <c r="K17" s="10">
-        <v>0</v>
-      </c>
-      <c r="L17" s="10">
-        <v>316591.67</v>
-      </c>
-      <c r="M17" s="10">
-        <v>0</v>
-      </c>
-      <c r="N17" s="10">
-        <v>316591.67</v>
-      </c>
-      <c r="O17" s="5" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18" s="15"/>
-      <c r="B18" s="15"/>
-      <c r="C18" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="D18" s="15"/>
-      <c r="E18" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
-      <c r="H18" s="16">
-        <v>300000</v>
-      </c>
-      <c r="I18" s="16">
-        <v>33458.34</v>
-      </c>
-      <c r="J18" s="16">
-        <v>0</v>
-      </c>
-      <c r="K18" s="16">
-        <v>0</v>
-      </c>
-      <c r="L18" s="16">
-        <v>333458.34</v>
-      </c>
-      <c r="M18" s="16">
-        <v>0</v>
-      </c>
-      <c r="N18" s="16">
-        <v>333458.34</v>
-      </c>
-      <c r="O18" s="15"/>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" s="17" t="s">
+      <c r="D22" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="G22" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="H22" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="I22" s="8" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="21" ht="30" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="B21" s="7" t="s">
+      <c r="J22" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="C21" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="D21" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="E21" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F21" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G21" s="7" t="s">
+      <c r="K22" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="H21" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="I21" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="J21" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="K21" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="L21" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="M21" s="7" t="s">
+      <c r="L22" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="N21" s="7" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" s="18" t="s">
-        <v>77</v>
+      <c r="M22" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="N22" s="8" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" s="25" t="s">
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>